<commit_message>
Apply approved accommodations: Bronson Christmas, Kennedy Nov weekend, Oghenesume April
- MacNeille Dec: Bronson takes the Christmas NF week 12/20-25 (approved by PD);
  MacNeille no Christmas nights + short call on NYE 12/31 (2 Q4 gaps).
- Kennedy Nov: enabled KEN_SWAP_DAYS (nights 11/1-5, off 11/7-8 weekend);
  Fri 11/6 handed to Chiasson so he does a light short call and can travel.
  Thanksgiving 11/26 already off. Friday ripple lands on Mullins (non-LSH).
- Oghenesume April: 4/10-11 weekend off (freed the 4/11 Sunday long call);
  4/9 & 4/12 stay short call (Thursday-only rule blocks full weekday days off).

All accommodation costs are documented Q4/coupling exceptions, landing on
non-LSH interns wherever possible. Regenerated full-year yearbook HTML +
monthly xlsx from the swapped schedule. Updated ACCOMMODATIONS.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_December_2026.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_December_2026.xlsx
@@ -521,12 +521,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE, SHETTY</t>
+          <t>BRONSON, SHETTY</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE, BRONSON</t>
+          <t>BRONSON, MACNEILLE</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -596,12 +596,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE, SHETTY</t>
+          <t>BRONSON, SHETTY</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -642,13 +642,13 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -668,12 +668,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>VILLANUEVA, MACNEILLE</t>
+          <t>VILLANUEVA, BRONSON</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -693,12 +693,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>VIVEKANANDAN, MACNEILLE</t>
+          <t>VIVEKANANDAN, BRONSON</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -768,12 +768,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>VIVEKANANDAN, MACNEILLE</t>
+          <t>VIVEKANANDAN, BRONSON</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -788,13 +788,13 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>MACNEILLE  (24H)</t>
+          <t>BRONSON  (24H)</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE, SALAM</t>
+          <t>BRONSON, SALAM</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>BRONSON, SALAM</t>
+          <t>MACNEILLE, SALAM</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>BRONSON, MACNEILLE</t>
+          <t>MACNEILLE, BRONSON</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -905,12 +905,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
+          <t>MACNEILLE</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
           <t>BRONSON</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -930,12 +930,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>BRONSON, SALAM</t>
+          <t>MACNEILLE, SALAM</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -976,13 +976,13 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
     </row>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>SALAM, BRONSON</t>
+          <t>SALAM, MACNEILLE</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>FARZEELA, BRONSON</t>
+          <t>FARZEELA, MACNEILLE</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
     </row>
@@ -1047,17 +1047,17 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
+          <t>MACNEILLE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>FARZEELA, SALAM</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
           <t>BRONSON</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>FARZEELA, SALAM</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>MACNEILLE</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
     </row>
@@ -1102,12 +1102,12 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>FARZEELA, BRONSON</t>
+          <t>FARZEELA, MACNEILLE</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
     </row>
@@ -1122,13 +1122,13 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>BRONSON  (24H)</t>
+          <t>MACNEILLE  (24H)</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>MACNEILLE</t>
+          <t>BRONSON</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>BRONSON</t>
+          <t>MACNEILLE</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">

</xml_diff>